<commit_message>
[update] 데이터 드리븐을 통한 Player, enemy, Bullit 초기화 및 Instantiate
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/WJBullit.xlsx
+++ b/JsonConverter/ExcelFiles/WJBullit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\WJMainProject2D\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82632469-BF8B-49F0-8E69-8D3419F1E4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C436D75-C81F-4C77-8B81-141EF9586F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4020" yWindow="1680" windowWidth="21270" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32505" yWindow="3765" windowWidth="21270" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WJTable_Bullit" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>(name)</t>
   </si>
@@ -78,11 +78,15 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>4f</t>
+    <t>_path</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>3f</t>
+    <t>string</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Prefabs/2D/Bullit</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -196,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -221,6 +225,9 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -445,7 +452,7 @@
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="19.5703125" customWidth="1"/>
     <col min="3" max="5" width="15.85546875" customWidth="1"/>
-    <col min="6" max="6" width="18.28515625" customWidth="1"/>
+    <col min="6" max="7" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" customHeight="1">
@@ -457,6 +464,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -477,6 +485,9 @@
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -497,6 +508,9 @@
       <c r="F3" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="4" spans="1:14" ht="15.75" customHeight="1">
       <c r="A4" s="4" t="s">
@@ -508,16 +522,18 @@
       <c r="C4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="12">
         <v>10</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="3"/>
+      <c r="E4" s="12">
+        <v>4</v>
+      </c>
+      <c r="F4" s="12">
+        <v>3</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>16</v>
+      </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
@@ -533,7 +549,7 @@
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="5"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -549,7 +565,7 @@
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
-      <c r="G6" s="3"/>
+      <c r="G6" s="5"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -565,7 +581,7 @@
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
-      <c r="G7" s="3"/>
+      <c r="G7" s="4"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -581,7 +597,7 @@
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
-      <c r="G8" s="3"/>
+      <c r="G8" s="6"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
@@ -597,7 +613,7 @@
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
-      <c r="G9" s="3"/>
+      <c r="G9" s="6"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -613,7 +629,7 @@
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
-      <c r="G10" s="3"/>
+      <c r="G10" s="7"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
@@ -629,7 +645,7 @@
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
-      <c r="G11" s="3"/>
+      <c r="G11" s="7"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
@@ -645,7 +661,7 @@
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
-      <c r="G12" s="3"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
@@ -661,7 +677,7 @@
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="3"/>
+      <c r="G13" s="4"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
@@ -677,7 +693,7 @@
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
-      <c r="G14" s="3"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
@@ -693,7 +709,7 @@
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
-      <c r="G15" s="3"/>
+      <c r="G15" s="7"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
@@ -709,172 +725,192 @@
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G16" s="8"/>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" customHeight="1">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" customHeight="1">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G18" s="9"/>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" customHeight="1">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" customHeight="1">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" customHeight="1">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" customHeight="1">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G22" s="9"/>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" customHeight="1">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
-    </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" customHeight="1">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" customHeight="1">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
-    </row>
-    <row r="26" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" customHeight="1">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
-    </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" ht="15.75" customHeight="1">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
-    </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G27" s="10"/>
+    </row>
+    <row r="28" spans="1:7" ht="15.75" customHeight="1">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
-    </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" ht="15.75" customHeight="1">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
-    </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G29" s="10"/>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" customHeight="1">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
-    </row>
-    <row r="31" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" ht="15.75" customHeight="1">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
-    </row>
-    <row r="32" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G31" s="10"/>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" customHeight="1">
       <c r="A32" s="11"/>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
       <c r="E32" s="11"/>
       <c r="F32" s="11"/>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G32" s="11"/>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" customHeight="1">
       <c r="A33" s="11"/>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
       <c r="D33" s="11"/>
       <c r="E33" s="11"/>
       <c r="F33" s="11"/>
-    </row>
-    <row r="34" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G33" s="11"/>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" customHeight="1">
       <c r="A34" s="11"/>
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
       <c r="E34" s="11"/>
       <c r="F34" s="11"/>
-    </row>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G34" s="11"/>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" customHeight="1">
       <c r="A35" s="11"/>
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
-    </row>
-    <row r="36" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="37" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="38" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="39" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="40" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="41" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="43" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="44" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="45" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="46" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="47" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="48" spans="1:6" ht="15.75" customHeight="1"/>
+      <c r="G35" s="11"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="37" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="38" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="39" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="40" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="41" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="42" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="43" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="44" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="45" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="46" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="47" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
[update] MeleeAtk 풀링 구현 완료
Bullit보다 개수가 많이 필요하지 않아 10개로 잡고 MeleeAtk 오브젝트(프리팹)만 보관하는 리스트 생성
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/WJBullit.xlsx
+++ b/JsonConverter/ExcelFiles/WJBullit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\WJMainProject2D\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD537BE-70FA-4EC6-866D-ED2FBD67FCB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007454BC-516F-44FD-B588-DAD4AEB4247B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1425" yWindow="2655" windowWidth="15345" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9900" yWindow="2985" windowWidth="17115" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WJTable_Bullit" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t>(name)</t>
   </si>
@@ -145,6 +145,26 @@
   </si>
   <si>
     <t>Icon/ArrowIcon</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Melee_Base_1</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>휘두르기</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Melee_Base_1_Lv1,Melee_Base_1_Lv2,Melee_Base_1_Lv3</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Icon/MeleeAtkIcon</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>가장 가까운 적에게 짧은 근접공격을 수행한다. 또한 살짝 뒤로 밀어낸다.</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -642,12 +662,24 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
+      <c r="A7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>

</xml_diff>